<commit_message>
data(week 20): real W20 inventory + corrected other-channels sales for W15-W20
- Replaced Week 20 inventory placeholder copies with real per-brand
  snapshots (Audio_Array, Nexlev, Tonor, WM); Fossil still pending
- Updated other_channels.xlsx for Audio_Array + Nexlev across W15-W20
  with corrected channel rosters (CRED_B2C added in W15-W16, POP one-off
  in W17, BI Worldwide drops ~95% in W20)
- Re-ran inventory_model_snapshot, inventory_snapshot_etl, sales_auto_etl,
  build_ai_context — all downstream outputs refreshed

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/raw/sales/Week 15/Audio_Array/other_channels.xlsx
+++ b/data/raw/sales/Week 15/Audio_Array/other_channels.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Other computers\My Laptop\D\Nitesh\Weekly Report - B2B + B2C\FastAPI\data\raw\sales\Week 15\Audio_Array\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F7EFD23-5EFA-46BF-9FD6-B55B3F425914}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA36916C-D823-4818-BAF3-BFA396AB6BBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="D2C - Audio Array" sheetId="4" r:id="rId1"/>
@@ -1249,7 +1249,7 @@
   <numFmts count="1">
     <numFmt numFmtId="8" formatCode="&quot;₹&quot;\ #,##0.00;[Red]&quot;₹&quot;\ \-#,##0.00"/>
   </numFmts>
-  <fonts count="13" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1310,12 +1310,6 @@
       <family val="2"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
@@ -1325,11 +1319,13 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="6">
@@ -1415,7 +1411,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1484,17 +1480,8 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1502,7 +1489,7 @@
     <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1511,19 +1498,19 @@
     <xf numFmtId="1" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -3222,7 +3209,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
-  <dimension ref="A1:W923"/>
+  <dimension ref="A1:W916"/>
   <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.109375" customWidth="1"/>
@@ -3272,142 +3259,142 @@
       <c r="W1" s="9"/>
     </row>
     <row r="2" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="26" t="s">
-        <v>381</v>
-      </c>
-      <c r="B2" s="27" t="s">
+      <c r="A2" t="s">
+        <v>381</v>
+      </c>
+      <c r="B2" t="s">
         <v>21</v>
       </c>
-      <c r="C2" s="27" t="s">
+      <c r="C2" t="s">
         <v>23</v>
       </c>
-      <c r="D2" s="27" t="s">
+      <c r="D2" t="s">
         <v>22</v>
       </c>
-      <c r="E2" s="28">
+      <c r="E2">
         <v>2</v>
       </c>
-      <c r="F2" s="29">
-        <v>8642.3700000000008</v>
+      <c r="F2">
+        <v>8642</v>
       </c>
     </row>
     <row r="3" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="26" t="s">
-        <v>381</v>
-      </c>
-      <c r="B3" s="27" t="s">
+      <c r="A3" t="s">
+        <v>381</v>
+      </c>
+      <c r="B3" t="s">
         <v>197</v>
       </c>
-      <c r="C3" s="27" t="s">
+      <c r="C3" t="s">
         <v>199</v>
       </c>
-      <c r="D3" s="27" t="s">
+      <c r="D3" t="s">
         <v>198</v>
       </c>
-      <c r="E3" s="28">
+      <c r="E3">
         <v>21</v>
       </c>
-      <c r="F3" s="29">
-        <v>33795.760000000002</v>
+      <c r="F3">
+        <v>33796</v>
       </c>
     </row>
     <row r="4" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="26" t="s">
-        <v>381</v>
-      </c>
-      <c r="B4" s="27" t="s">
+      <c r="A4" t="s">
+        <v>381</v>
+      </c>
+      <c r="B4" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="27" t="s">
+      <c r="C4" t="s">
         <v>15</v>
       </c>
-      <c r="D4" s="27" t="s">
+      <c r="D4" t="s">
         <v>14</v>
       </c>
-      <c r="E4" s="28">
+      <c r="E4">
         <v>5</v>
       </c>
-      <c r="F4" s="29">
-        <v>11266.95</v>
+      <c r="F4">
+        <v>11267</v>
       </c>
     </row>
     <row r="5" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="26" t="s">
-        <v>381</v>
-      </c>
-      <c r="B5" s="27" t="s">
+      <c r="A5" t="s">
+        <v>381</v>
+      </c>
+      <c r="B5" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="27" t="s">
+      <c r="C5" t="s">
         <v>11</v>
       </c>
-      <c r="D5" s="27" t="s">
+      <c r="D5" t="s">
         <v>10</v>
       </c>
-      <c r="E5" s="28">
+      <c r="E5">
         <v>1</v>
       </c>
-      <c r="F5" s="29">
-        <v>4066.95</v>
+      <c r="F5">
+        <v>4067</v>
       </c>
     </row>
     <row r="6" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="26" t="s">
-        <v>381</v>
-      </c>
-      <c r="B6" s="27" t="s">
+      <c r="A6" t="s">
+        <v>381</v>
+      </c>
+      <c r="B6" t="s">
         <v>29</v>
       </c>
-      <c r="C6" s="27" t="s">
+      <c r="C6" t="s">
         <v>31</v>
       </c>
-      <c r="D6" s="27" t="s">
+      <c r="D6" t="s">
         <v>30</v>
       </c>
-      <c r="E6" s="28">
+      <c r="E6">
         <v>4</v>
       </c>
-      <c r="F6" s="29">
-        <v>11925.42</v>
+      <c r="F6">
+        <v>11925</v>
       </c>
     </row>
     <row r="7" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="26" t="s">
-        <v>381</v>
-      </c>
-      <c r="B7" s="27" t="s">
+      <c r="A7" t="s">
+        <v>381</v>
+      </c>
+      <c r="B7" t="s">
         <v>315</v>
       </c>
-      <c r="C7" s="27" t="s">
+      <c r="C7" t="s">
         <v>317</v>
       </c>
-      <c r="D7" s="27" t="s">
+      <c r="D7" t="s">
         <v>316</v>
       </c>
-      <c r="E7" s="28">
+      <c r="E7">
         <v>3</v>
       </c>
-      <c r="F7" s="29">
-        <v>4022.88</v>
+      <c r="F7">
+        <v>4023</v>
       </c>
     </row>
     <row r="8" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="26" t="s">
-        <v>381</v>
-      </c>
-      <c r="B8" s="27" t="s">
+      <c r="A8" t="s">
+        <v>381</v>
+      </c>
+      <c r="B8" t="s">
         <v>77</v>
       </c>
-      <c r="C8" s="27" t="s">
+      <c r="C8" t="s">
         <v>79</v>
       </c>
-      <c r="D8" s="27" t="s">
+      <c r="D8" t="s">
         <v>78</v>
       </c>
-      <c r="E8" s="28">
+      <c r="E8">
         <v>0</v>
       </c>
-      <c r="F8" s="29">
+      <c r="F8">
         <v>0</v>
       </c>
     </row>
@@ -4319,13 +4306,6 @@
     <row r="914" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="915" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="916" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="917" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="918" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="919" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="920" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="921" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="922" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="923" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
@@ -7009,10 +6989,10 @@
       <c r="A2" s="21" t="s">
         <v>287</v>
       </c>
-      <c r="B2" s="30" t="s">
+      <c r="B2" s="27" t="s">
         <v>289</v>
       </c>
-      <c r="C2" s="31" t="s">
+      <c r="C2" s="28" t="s">
         <v>288</v>
       </c>
       <c r="D2" s="21">
@@ -7021,30 +7001,30 @@
       <c r="E2" s="21">
         <v>3048</v>
       </c>
-      <c r="F2" s="32" t="s">
-        <v>381</v>
-      </c>
-      <c r="G2" s="30" t="s">
+      <c r="F2" s="29" t="s">
+        <v>381</v>
+      </c>
+      <c r="G2" s="27" t="s">
         <v>388</v>
       </c>
     </row>
     <row r="3" spans="1:25" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="33" t="s">
+      <c r="A3" s="30" t="s">
         <v>97</v>
       </c>
       <c r="B3" s="21" t="s">
         <v>99</v>
       </c>
-      <c r="C3" s="28" t="s">
+      <c r="C3" s="26" t="s">
         <v>98</v>
       </c>
-      <c r="D3" s="28">
+      <c r="D3" s="26">
         <v>2</v>
       </c>
-      <c r="E3" s="34">
+      <c r="E3" s="31">
         <v>5695</v>
       </c>
-      <c r="F3" s="35" t="s">
+      <c r="F3" s="32" t="s">
         <v>381</v>
       </c>
       <c r="G3" s="21" t="s">
@@ -7052,22 +7032,22 @@
       </c>
     </row>
     <row r="4" spans="1:25" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="33" t="s">
+      <c r="A4" s="30" t="s">
         <v>9</v>
       </c>
       <c r="B4" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="28" t="s">
+      <c r="C4" s="26" t="s">
         <v>10</v>
       </c>
-      <c r="D4" s="28">
+      <c r="D4" s="26">
         <v>2</v>
       </c>
-      <c r="E4" s="34">
+      <c r="E4" s="31">
         <v>5636</v>
       </c>
-      <c r="F4" s="35" t="s">
+      <c r="F4" s="32" t="s">
         <v>381</v>
       </c>
       <c r="G4" s="21" t="s">
@@ -7075,22 +7055,22 @@
       </c>
     </row>
     <row r="5" spans="1:25" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="33" t="s">
+      <c r="A5" s="30" t="s">
         <v>263</v>
       </c>
       <c r="B5" s="21" t="s">
         <v>265</v>
       </c>
-      <c r="C5" s="28" t="s">
+      <c r="C5" s="26" t="s">
         <v>264</v>
       </c>
-      <c r="D5" s="28">
+      <c r="D5" s="26">
         <v>2</v>
       </c>
-      <c r="E5" s="34">
+      <c r="E5" s="31">
         <v>4331</v>
       </c>
-      <c r="F5" s="35" t="s">
+      <c r="F5" s="32" t="s">
         <v>381</v>
       </c>
       <c r="G5" s="21" t="s">
@@ -7098,22 +7078,22 @@
       </c>
     </row>
     <row r="6" spans="1:25" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="33" t="s">
+      <c r="A6" s="30" t="s">
         <v>109</v>
       </c>
       <c r="B6" s="21" t="s">
         <v>111</v>
       </c>
-      <c r="C6" s="28" t="s">
+      <c r="C6" s="26" t="s">
         <v>110</v>
       </c>
-      <c r="D6" s="28">
+      <c r="D6" s="26">
         <v>2</v>
       </c>
-      <c r="E6" s="34">
+      <c r="E6" s="31">
         <v>5576</v>
       </c>
-      <c r="F6" s="35" t="s">
+      <c r="F6" s="32" t="s">
         <v>381</v>
       </c>
       <c r="G6" s="21" t="s">
@@ -7121,22 +7101,22 @@
       </c>
     </row>
     <row r="7" spans="1:25" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="33" t="s">
+      <c r="A7" s="30" t="s">
         <v>233</v>
       </c>
       <c r="B7" s="21" t="s">
         <v>235</v>
       </c>
-      <c r="C7" s="28" t="s">
+      <c r="C7" s="26" t="s">
         <v>234</v>
       </c>
-      <c r="D7" s="28">
+      <c r="D7" s="26">
         <v>2</v>
       </c>
-      <c r="E7" s="34">
+      <c r="E7" s="31">
         <v>5814</v>
       </c>
-      <c r="F7" s="35" t="s">
+      <c r="F7" s="32" t="s">
         <v>381</v>
       </c>
       <c r="G7" s="21" t="s">
@@ -7144,22 +7124,22 @@
       </c>
     </row>
     <row r="8" spans="1:25" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="33" t="s">
+      <c r="A8" s="30" t="s">
         <v>133</v>
       </c>
       <c r="B8" s="21" t="s">
         <v>135</v>
       </c>
-      <c r="C8" s="28" t="s">
+      <c r="C8" s="26" t="s">
         <v>134</v>
       </c>
-      <c r="D8" s="28">
+      <c r="D8" s="26">
         <v>2</v>
       </c>
-      <c r="E8" s="28">
+      <c r="E8" s="26">
         <v>4153</v>
       </c>
-      <c r="F8" s="35" t="s">
+      <c r="F8" s="32" t="s">
         <v>381</v>
       </c>
       <c r="G8" s="21" t="s">
@@ -7167,22 +7147,22 @@
       </c>
     </row>
     <row r="9" spans="1:25" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="33" t="s">
+      <c r="A9" s="30" t="s">
         <v>373</v>
       </c>
       <c r="B9" s="21" t="s">
         <v>375</v>
       </c>
-      <c r="C9" s="28" t="s">
+      <c r="C9" s="26" t="s">
         <v>374</v>
       </c>
-      <c r="D9" s="28">
+      <c r="D9" s="26">
         <v>2</v>
       </c>
-      <c r="E9" s="28">
+      <c r="E9" s="26">
         <v>4746</v>
       </c>
-      <c r="F9" s="35" t="s">
+      <c r="F9" s="32" t="s">
         <v>381</v>
       </c>
       <c r="G9" s="21" t="s">
@@ -7190,22 +7170,22 @@
       </c>
     </row>
     <row r="10" spans="1:25" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="33" t="s">
+      <c r="A10" s="30" t="s">
         <v>365</v>
       </c>
       <c r="B10" s="21" t="s">
         <v>367</v>
       </c>
-      <c r="C10" s="28" t="s">
+      <c r="C10" s="26" t="s">
         <v>366</v>
       </c>
-      <c r="D10" s="28">
+      <c r="D10" s="26">
         <v>2</v>
       </c>
-      <c r="E10" s="28">
+      <c r="E10" s="26">
         <v>2542</v>
       </c>
-      <c r="F10" s="35" t="s">
+      <c r="F10" s="32" t="s">
         <v>381</v>
       </c>
       <c r="G10" s="21" t="s">
@@ -7213,22 +7193,22 @@
       </c>
     </row>
     <row r="11" spans="1:25" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="33" t="s">
+      <c r="A11" s="30" t="s">
         <v>125</v>
       </c>
       <c r="B11" s="21" t="s">
         <v>127</v>
       </c>
-      <c r="C11" s="28" t="s">
+      <c r="C11" s="26" t="s">
         <v>126</v>
       </c>
-      <c r="D11" s="28">
+      <c r="D11" s="26">
         <v>2</v>
       </c>
-      <c r="E11" s="28">
+      <c r="E11" s="26">
         <v>5085</v>
       </c>
-      <c r="F11" s="35" t="s">
+      <c r="F11" s="32" t="s">
         <v>381</v>
       </c>
       <c r="G11" s="21" t="s">
@@ -7236,22 +7216,22 @@
       </c>
     </row>
     <row r="12" spans="1:25" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="33" t="s">
+      <c r="A12" s="30" t="s">
         <v>17</v>
       </c>
       <c r="B12" s="21" t="s">
         <v>19</v>
       </c>
-      <c r="C12" s="28" t="s">
+      <c r="C12" s="26" t="s">
         <v>18</v>
       </c>
-      <c r="D12" s="28">
+      <c r="D12" s="26">
         <v>2</v>
       </c>
-      <c r="E12" s="28">
+      <c r="E12" s="26">
         <v>10441</v>
       </c>
-      <c r="F12" s="35" t="s">
+      <c r="F12" s="32" t="s">
         <v>381</v>
       </c>
       <c r="G12" s="21" t="s">
@@ -7259,22 +7239,22 @@
       </c>
     </row>
     <row r="13" spans="1:25" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="33" t="s">
+      <c r="A13" s="30" t="s">
         <v>77</v>
       </c>
       <c r="B13" s="21" t="s">
         <v>79</v>
       </c>
-      <c r="C13" s="28" t="s">
+      <c r="C13" s="26" t="s">
         <v>78</v>
       </c>
-      <c r="D13" s="28">
+      <c r="D13" s="26">
         <v>2</v>
       </c>
-      <c r="E13" s="28">
+      <c r="E13" s="26">
         <v>1525</v>
       </c>
-      <c r="F13" s="35" t="s">
+      <c r="F13" s="32" t="s">
         <v>381</v>
       </c>
       <c r="G13" s="21" t="s">
@@ -7282,22 +7262,22 @@
       </c>
     </row>
     <row r="14" spans="1:25" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="33" t="s">
+      <c r="A14" s="30" t="s">
         <v>255</v>
       </c>
       <c r="B14" s="21" t="s">
         <v>257</v>
       </c>
-      <c r="C14" s="28" t="s">
+      <c r="C14" s="26" t="s">
         <v>390</v>
       </c>
-      <c r="D14" s="28">
+      <c r="D14" s="26">
         <v>2</v>
       </c>
-      <c r="E14" s="34">
+      <c r="E14" s="31">
         <v>2542</v>
       </c>
-      <c r="F14" s="35" t="s">
+      <c r="F14" s="32" t="s">
         <v>381</v>
       </c>
       <c r="G14" s="21" t="s">
@@ -7305,22 +7285,22 @@
       </c>
     </row>
     <row r="15" spans="1:25" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="33" t="s">
+      <c r="A15" s="30" t="s">
         <v>129</v>
       </c>
       <c r="B15" s="21" t="s">
         <v>131</v>
       </c>
-      <c r="C15" s="28" t="s">
+      <c r="C15" s="26" t="s">
         <v>391</v>
       </c>
-      <c r="D15" s="28">
+      <c r="D15" s="26">
         <v>2</v>
       </c>
-      <c r="E15" s="34">
+      <c r="E15" s="31">
         <v>2542</v>
       </c>
-      <c r="F15" s="35" t="s">
+      <c r="F15" s="32" t="s">
         <v>381</v>
       </c>
       <c r="G15" s="21" t="s">
@@ -7328,22 +7308,22 @@
       </c>
     </row>
     <row r="16" spans="1:25" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="33" t="s">
+      <c r="A16" s="30" t="s">
         <v>279</v>
       </c>
       <c r="B16" s="21" t="s">
         <v>281</v>
       </c>
-      <c r="C16" s="28" t="s">
+      <c r="C16" s="26" t="s">
         <v>280</v>
       </c>
-      <c r="D16" s="28">
+      <c r="D16" s="26">
         <v>2</v>
       </c>
-      <c r="E16" s="34">
+      <c r="E16" s="31">
         <v>3814</v>
       </c>
-      <c r="F16" s="35" t="s">
+      <c r="F16" s="32" t="s">
         <v>381</v>
       </c>
       <c r="G16" s="21" t="s">
@@ -7351,22 +7331,22 @@
       </c>
     </row>
     <row r="17" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="33" t="s">
+      <c r="A17" s="30" t="s">
         <v>217</v>
       </c>
       <c r="B17" s="21" t="s">
         <v>219</v>
       </c>
-      <c r="C17" s="28" t="s">
+      <c r="C17" s="26" t="s">
         <v>218</v>
       </c>
-      <c r="D17" s="28">
+      <c r="D17" s="26">
         <v>2</v>
       </c>
-      <c r="E17" s="34">
+      <c r="E17" s="31">
         <v>2254</v>
       </c>
-      <c r="F17" s="35" t="s">
+      <c r="F17" s="32" t="s">
         <v>381</v>
       </c>
       <c r="G17" s="21" t="s">
@@ -7374,22 +7354,22 @@
       </c>
     </row>
     <row r="18" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="33" t="s">
+      <c r="A18" s="30" t="s">
         <v>319</v>
       </c>
       <c r="B18" s="21" t="s">
         <v>321</v>
       </c>
-      <c r="C18" s="28" t="s">
+      <c r="C18" s="26" t="s">
         <v>320</v>
       </c>
-      <c r="D18" s="28">
+      <c r="D18" s="26">
         <v>1</v>
       </c>
-      <c r="E18" s="34">
+      <c r="E18" s="31">
         <v>12458</v>
       </c>
-      <c r="F18" s="35" t="s">
+      <c r="F18" s="32" t="s">
         <v>381</v>
       </c>
       <c r="G18" s="21" t="s">
@@ -7397,22 +7377,22 @@
       </c>
     </row>
     <row r="19" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="33" t="s">
+      <c r="A19" s="30" t="s">
         <v>392</v>
       </c>
       <c r="B19" s="21" t="s">
         <v>393</v>
       </c>
-      <c r="C19" s="28" t="s">
+      <c r="C19" s="26" t="s">
         <v>394</v>
       </c>
-      <c r="D19" s="28">
+      <c r="D19" s="26">
         <v>1</v>
       </c>
-      <c r="E19" s="34">
+      <c r="E19" s="31">
         <v>12458</v>
       </c>
-      <c r="F19" s="35" t="s">
+      <c r="F19" s="32" t="s">
         <v>381</v>
       </c>
       <c r="G19" s="21" t="s">
@@ -7420,22 +7400,22 @@
       </c>
     </row>
     <row r="20" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="33" t="s">
+      <c r="A20" s="30" t="s">
         <v>395</v>
       </c>
       <c r="B20" s="21" t="s">
         <v>396</v>
       </c>
-      <c r="C20" s="28" t="s">
+      <c r="C20" s="26" t="s">
         <v>397</v>
       </c>
-      <c r="D20" s="28">
+      <c r="D20" s="26">
         <v>1</v>
       </c>
-      <c r="E20" s="34">
+      <c r="E20" s="31">
         <v>10085</v>
       </c>
-      <c r="F20" s="35" t="s">
+      <c r="F20" s="32" t="s">
         <v>381</v>
       </c>
       <c r="G20" s="21" t="s">
@@ -7443,22 +7423,22 @@
       </c>
     </row>
     <row r="21" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="33" t="s">
+      <c r="A21" s="30" t="s">
         <v>251</v>
       </c>
       <c r="B21" s="21" t="s">
         <v>253</v>
       </c>
-      <c r="C21" s="28" t="s">
+      <c r="C21" s="26" t="s">
         <v>252</v>
       </c>
-      <c r="D21" s="28">
+      <c r="D21" s="26">
         <v>2</v>
       </c>
-      <c r="E21" s="34">
+      <c r="E21" s="31">
         <v>5102</v>
       </c>
-      <c r="F21" s="35" t="s">
+      <c r="F21" s="32" t="s">
         <v>381</v>
       </c>
       <c r="G21" s="21" t="s">
@@ -7466,22 +7446,22 @@
       </c>
     </row>
     <row r="22" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="33" t="s">
+      <c r="A22" s="30" t="s">
         <v>357</v>
       </c>
       <c r="B22" s="21" t="s">
         <v>359</v>
       </c>
-      <c r="C22" s="28" t="s">
+      <c r="C22" s="26" t="s">
         <v>358</v>
       </c>
-      <c r="D22" s="28">
+      <c r="D22" s="26">
         <v>2</v>
       </c>
-      <c r="E22" s="34">
+      <c r="E22" s="31">
         <v>5102</v>
       </c>
-      <c r="F22" s="35" t="s">
+      <c r="F22" s="32" t="s">
         <v>381</v>
       </c>
       <c r="G22" s="21" t="s">
@@ -7489,22 +7469,22 @@
       </c>
     </row>
     <row r="23" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="33" t="s">
+      <c r="A23" s="30" t="s">
         <v>105</v>
       </c>
       <c r="B23" s="21" t="s">
         <v>107</v>
       </c>
-      <c r="C23" s="28" t="s">
+      <c r="C23" s="26" t="s">
         <v>106</v>
       </c>
-      <c r="D23" s="28">
+      <c r="D23" s="26">
         <v>2</v>
       </c>
-      <c r="E23" s="34">
+      <c r="E23" s="31">
         <v>7119</v>
       </c>
-      <c r="F23" s="35" t="s">
+      <c r="F23" s="32" t="s">
         <v>381</v>
       </c>
       <c r="G23" s="21" t="s">
@@ -7512,22 +7492,22 @@
       </c>
     </row>
     <row r="24" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="33" t="s">
+      <c r="A24" s="30" t="s">
         <v>221</v>
       </c>
       <c r="B24" s="21" t="s">
         <v>223</v>
       </c>
-      <c r="C24" s="28" t="s">
+      <c r="C24" s="26" t="s">
         <v>222</v>
       </c>
-      <c r="D24" s="28">
+      <c r="D24" s="26">
         <v>2</v>
       </c>
-      <c r="E24" s="34">
+      <c r="E24" s="31">
         <v>7119</v>
       </c>
-      <c r="F24" s="35" t="s">
+      <c r="F24" s="32" t="s">
         <v>381</v>
       </c>
       <c r="G24" s="21" t="s">
@@ -7535,22 +7515,22 @@
       </c>
     </row>
     <row r="25" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="36" t="s">
+      <c r="A25" s="33" t="s">
         <v>189</v>
       </c>
       <c r="B25" s="21" t="s">
         <v>189</v>
       </c>
-      <c r="C25" s="36" t="s">
+      <c r="C25" s="33" t="s">
         <v>190</v>
       </c>
-      <c r="D25" s="36">
+      <c r="D25" s="33">
         <v>10</v>
       </c>
       <c r="E25" s="22">
         <v>20762.71</v>
       </c>
-      <c r="F25" s="35" t="s">
+      <c r="F25" s="32" t="s">
         <v>381</v>
       </c>
       <c r="G25" s="21" t="s">
@@ -7558,25 +7538,25 @@
       </c>
     </row>
     <row r="26" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="38" t="s">
+      <c r="A26" s="35" t="s">
         <v>177</v>
       </c>
-      <c r="B26" s="37" t="s">
+      <c r="B26" s="34" t="s">
         <v>179</v>
       </c>
-      <c r="C26" s="39" t="s">
+      <c r="C26" s="36" t="s">
         <v>178</v>
       </c>
-      <c r="D26" s="38">
+      <c r="D26" s="35">
         <v>1</v>
       </c>
-      <c r="E26" s="38">
+      <c r="E26" s="35">
         <v>850</v>
       </c>
-      <c r="F26" s="35" t="s">
-        <v>381</v>
-      </c>
-      <c r="G26" s="37" t="s">
+      <c r="F26" s="32" t="s">
+        <v>381</v>
+      </c>
+      <c r="G26" s="34" t="s">
         <v>399</v>
       </c>
     </row>

</xml_diff>